<commit_message>
v2.1: GUI Polish — YAML view fixes, scrollbar, Schemas indent, converter examples, 400 sandbox params (builds 2.1.43-2.1.60)
</commit_message>
<xml_diff>
--- a/Templates Master/$index.xlsx
+++ b/Templates Master/$index.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\giuse\.gemini\antigravity\scratch\OASIS\Templates Master\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F4DC543-1202-425A-97A5-BFC4FA2419F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10114D8E-6604-45EF-A0FA-F942177FC671}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General Description" sheetId="1" r:id="rId1"/>
@@ -463,11 +463,30 @@
     <cellStyle name="Titolo 1" xfId="1" builtinId="16"/>
     <cellStyle name="Titolo 3" xfId="2" builtinId="18"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
     <dxf>
       <font>
         <b/>
+        <i/>
+        <strike val="0"/>
       </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -26736,8 +26755,8 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:A1048576">
-    <cfRule type="expression" dxfId="0" priority="2">
-      <formula>$B2 = ""</formula>
+    <cfRule type="expression" dxfId="1" priority="2">
+      <formula>AND($A2&lt;&gt;"",$B2="")</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>